<commit_message>
feat: update service catalog, logic integration and import templates
</commit_message>
<xml_diff>
--- a/data/mau-file-import/mau_import_dich_vu_khac.xlsx
+++ b/data/mau-file-import/mau_import_dich_vu_khac.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Tên dịch vụ</t>
+          <t>Mã dịch vụ</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>HCC</t>
+          <t>CT_LH</t>
         </is>
       </c>
       <c r="D2" s="4" t="n">
@@ -613,7 +613,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>TCBC</t>
+          <t>TK_TT</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
@@ -710,12 +710,12 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Tên dịch vụ</t>
+          <t>Mã dịch vụ</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Tên dịch vụ (Vd: HCC, TCBC, PPBL). Lưu ý: phải khớp với tên trong hệ thống.</t>
+          <t>Mã dịch vụ viết tắt (Vd: CT_LH, TK_TT, B2B...). Tra cứu mã dịch vụ chính xác tại file ma_tham_chieu.xlsx, sheet 'Nhóm dịch vụ', cột 'Mã dịch vụ (Dùng nạp file)'.</t>
         </is>
       </c>
     </row>

</xml_diff>